<commit_message>
Atualizacao automatica da planilha - 21/09/2026 17:18
</commit_message>
<xml_diff>
--- a/Pedidos_Manutencao.xlsx
+++ b/Pedidos_Manutencao.xlsx
@@ -588,7 +588,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>EM EXECUCAO</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -623,27 +623,39 @@
         </is>
       </c>
       <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>7289-1</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="Q2" t="inlineStr">
         <is>
           <t>SERGIO PRATES PEREIRA</t>
         </is>
       </c>
       <c r="R2" t="n">
-        <v>3210</v>
+        <v>3049.5</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>588.53000000</t>
+          <t>559.10000000</t>
         </is>
       </c>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="n">
-        <v>3798.53</v>
+        <v>3608.6</v>
       </c>
       <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>3608.60000000</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">

</xml_diff>